<commit_message>
[FIX] set "company_id" on contact's addresses (for sheet "company")
</commit_message>
<xml_diff>
--- a/product_import_helper/static/xls/product_import_helper_template.xlsx
+++ b/product_import_helper/static/xls/product_import_helper_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,11 +22,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="233">
   <si>
     <t xml:space="preserve">IDENTIFICATION</t>
   </si>
   <si>
+    <t xml:space="preserve">VARIANTS</t>
+  </si>
+  <si>
     <t xml:space="preserve">VENTES</t>
   </si>
   <si>
@@ -78,6 +81,21 @@
     <t xml:space="preserve">Suivi en stock</t>
   </si>
   <si>
+    <t xml:space="preserve">Référence (template)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attribut 1 (remplacer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attribut 2 (remplacer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attribut 3 (remplacer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attribut 4 (remplacer)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Peut être vendu</t>
   </si>
   <si>
@@ -237,6 +255,21 @@
     <t xml:space="preserve">is_storable</t>
   </si>
   <si>
+    <t xml:space="preserve">default_code_tmpl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attr_Name1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attr_Name2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attr_Name3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">…</t>
+  </si>
+  <si>
     <t xml:space="preserve">sale_ok</t>
   </si>
   <si>
@@ -379,6 +412,18 @@
   </si>
   <si>
     <t xml:space="preserve">TRUE,FALSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plat</t>
   </si>
   <si>
     <t xml:space="preserve">order,delivery</t>
@@ -550,7 +595,7 @@
     <t xml:space="preserve">Nom du produit.</t>
   </si>
   <si>
-    <t xml:space="preserve">Référence de l’article.
+    <t xml:space="preserve">Référence de l’article (si “default_code_tpl” est utilisé : indiquer ici la référence du variant)
 L’import alerte concernant les doublons.</t>
   </si>
   <si>
@@ -577,6 +622,119 @@
   <si>
     <t xml:space="preserve">Uniquement si “type” = “consu” (biens)
 Si le niveau de stock est suivi en quantité (inventaire, incrément à l’achat, décrément à la vente ou à la consommation dans un process de fabrication, …)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Si renseigné, l’import bascule en mode “gestion des variants” et la référence </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">default_code_tmpl</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> désigne la référence de l’article de base (le “template”).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Dans “</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">attr_Name1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">”, remplacer “</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Name1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">” par le </t>
+    </r>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">nom</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> des attributs dans le menu “Inventaire &gt; Configuration &gt; Attributs”. Ajouter ou supprimer des colonnes pour ajouter des attributs ou correspondre à ceux déjà existant. Ainsi, dans ce fichier :
+- le nom de la colonne correspond aux noms des attributs (i.e. les “axes” de valeurs de variants)
+- le contenu des cellules du tableau correspond aux valeurs possibles des attributs. Elles seront créées si elle n’existent pas déjà</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Idem</t>
   </si>
   <si>
     <t xml:space="preserve">Si sélectionnable dans les devis, commandes et factures clients.
@@ -1162,7 +1320,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1173,6 +1331,12 @@
       <patternFill patternType="solid">
         <fgColor theme="6"/>
         <bgColor rgb="FF158466"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE16173"/>
+        <bgColor rgb="FFFF8000"/>
       </patternFill>
     </fill>
     <fill>
@@ -1196,7 +1360,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF8000"/>
-        <bgColor rgb="FFFF8080"/>
+        <bgColor rgb="FFE16173"/>
       </patternFill>
     </fill>
     <fill>
@@ -1246,7 +1410,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1263,42 +1427,46 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1316,18 +1484,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1395,7 +1567,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1419,27 +1591,27 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1487,7 +1659,7 @@
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FFE16173"/>
       <rgbColor rgb="FF2A6099"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
@@ -1704,8 +1876,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD6"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:BE6"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.92"/>
@@ -1717,43 +1889,45 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="19.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="16.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="19.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="28.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="17.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="25.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="21.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="21.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="19.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="19.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="18.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="24.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="25.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="21.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="23" style="1" width="19.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="25.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="23.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="14.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="15.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="1" width="20.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="15.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="31" style="1" width="25.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="29.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="15.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="35" style="1" width="25.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="37" style="1" width="23.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="19.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="17.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="24.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="23.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="13.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="17.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="21.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="17.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="16.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="49" style="1" width="19.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="50" min="50" style="1" width="19.11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16379" min="51" style="1" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="19.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="12" style="1" width="20.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="19.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="28.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="17.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="25.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="21.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="21.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="19.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="19.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="18.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="24.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="25.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="21.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="28" style="1" width="19.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="1" width="25.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="1" width="23.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="1" width="14.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="20.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="1" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="36" style="1" width="25.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="29.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="15.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="40" style="1" width="25.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="42" style="1" width="23.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="19.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="17.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="24.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="23.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="13.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="49" style="1" width="17.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="50" min="50" style="1" width="21.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="51" min="51" style="1" width="17.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="52" style="1" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="53" min="53" style="1" width="16.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="54" min="54" style="1" width="19.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="55" min="55" style="1" width="19.11"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="56" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1775,680 +1949,733 @@
       <c r="M1" s="4"/>
       <c r="N1" s="4"/>
       <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>2</v>
       </c>
+      <c r="Q1" s="5"/>
       <c r="R1" s="5"/>
       <c r="S1" s="5"/>
-      <c r="T1" s="6" t="s">
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="U1" s="7"/>
-      <c r="V1" s="7"/>
-      <c r="W1" s="7"/>
-      <c r="X1" s="7"/>
-      <c r="Y1" s="7"/>
-      <c r="Z1" s="7"/>
-      <c r="AA1" s="6" t="s">
+      <c r="W1" s="6"/>
+      <c r="X1" s="6"/>
+      <c r="Y1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="AB1" s="7"/>
-      <c r="AC1" s="7"/>
-      <c r="AD1" s="7"/>
-      <c r="AE1" s="7"/>
-      <c r="AF1" s="7"/>
-      <c r="AG1" s="8" t="s">
+      <c r="Z1" s="8"/>
+      <c r="AA1" s="8"/>
+      <c r="AB1" s="8"/>
+      <c r="AC1" s="8"/>
+      <c r="AD1" s="8"/>
+      <c r="AE1" s="8"/>
+      <c r="AF1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="AH1" s="9"/>
+      <c r="AG1" s="8"/>
+      <c r="AH1" s="8"/>
       <c r="AI1" s="8"/>
-      <c r="AJ1" s="9"/>
-      <c r="AK1" s="9"/>
-      <c r="AL1" s="10" t="s">
+      <c r="AJ1" s="8"/>
+      <c r="AK1" s="8"/>
+      <c r="AL1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="AM1" s="11"/>
-      <c r="AN1" s="12" t="s">
+      <c r="AM1" s="10"/>
+      <c r="AN1" s="9"/>
+      <c r="AO1" s="10"/>
+      <c r="AP1" s="10"/>
+      <c r="AQ1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="AO1" s="12"/>
-      <c r="AP1" s="12"/>
-      <c r="AQ1" s="12"/>
       <c r="AR1" s="12"/>
-      <c r="AS1" s="12"/>
-      <c r="AT1" s="12"/>
-      <c r="AU1" s="12"/>
-      <c r="AV1" s="12"/>
-      <c r="AW1" s="12"/>
-      <c r="AX1" s="12"/>
+      <c r="AS1" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="AT1" s="13"/>
+      <c r="AU1" s="13"/>
+      <c r="AV1" s="13"/>
+      <c r="AW1" s="13"/>
+      <c r="AX1" s="13"/>
       <c r="AY1" s="13"/>
       <c r="AZ1" s="13"/>
-      <c r="XEZ1" s="13"/>
-      <c r="XFA1" s="13"/>
-      <c r="XFB1" s="13"/>
-      <c r="XFC1" s="13"/>
-      <c r="XFD1" s="13"/>
-    </row>
-    <row r="2" s="14" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="15" t="s">
+      <c r="BA1" s="13"/>
+      <c r="BB1" s="13"/>
+      <c r="BC1" s="13"/>
+      <c r="BD1" s="14"/>
+      <c r="BE1" s="14"/>
+    </row>
+    <row r="2" s="15" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="D2" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="E2" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="F2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="G2" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="H2" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="I2" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="J2" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="K2" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="16" t="s">
+      <c r="L2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="N2" s="16" t="s">
+      <c r="M2" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="O2" s="16" t="s">
+      <c r="N2" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="P2" s="16" t="s">
+      <c r="O2" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="17" t="s">
+      <c r="P2" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="17" t="s">
+      <c r="Q2" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="S2" s="17" t="s">
+      <c r="R2" s="18" t="s">
         <v>26</v>
       </c>
+      <c r="S2" s="18" t="s">
+        <v>27</v>
+      </c>
       <c r="T2" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U2" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="V2" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="W2" s="18" t="s">
+      <c r="V2" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="X2" s="18" t="s">
+      <c r="W2" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="Y2" s="18" t="s">
+      <c r="X2" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="Z2" s="18" t="s">
+      <c r="Y2" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="AA2" s="18" t="s">
+      <c r="Z2" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="AB2" s="18" t="s">
+      <c r="AA2" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="AC2" s="18" t="s">
+      <c r="AB2" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="AD2" s="18" t="s">
+      <c r="AC2" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="AE2" s="18" t="s">
+      <c r="AD2" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="AF2" s="18" t="s">
+      <c r="AE2" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="AG2" s="19" t="s">
+      <c r="AF2" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="AH2" s="19" t="s">
+      <c r="AG2" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="AI2" s="19" t="s">
+      <c r="AH2" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="AJ2" s="19" t="s">
+      <c r="AI2" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="AK2" s="19" t="s">
+      <c r="AJ2" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="AL2" s="11" t="s">
+      <c r="AK2" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="AM2" s="11" t="s">
+      <c r="AL2" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="AN2" s="20" t="s">
+      <c r="AM2" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="AO2" s="20" t="s">
+      <c r="AN2" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="AP2" s="20" t="s">
+      <c r="AO2" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="AQ2" s="20" t="s">
+      <c r="AP2" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="AR2" s="20" t="s">
+      <c r="AQ2" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="AS2" s="20" t="s">
+      <c r="AR2" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="AT2" s="20" t="s">
+      <c r="AS2" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="AU2" s="20" t="s">
+      <c r="AT2" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="AV2" s="20" t="s">
+      <c r="AU2" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="AW2" s="20" t="s">
+      <c r="AV2" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="AX2" s="20" t="s">
+      <c r="AW2" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="AY2" s="13"/>
-      <c r="AZ2" s="13"/>
-      <c r="XFC2" s="1"/>
-      <c r="XFD2" s="1"/>
-    </row>
-    <row r="3" s="21" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
+      <c r="AX2" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="AY2" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" s="23" t="s">
+      <c r="AZ2" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="F3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="G3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="H3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="I3" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="J3" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="K3" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="L3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="M3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="N3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="O3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="P3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q3" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="R3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="S3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="T3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="U3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="V3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="W3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="X3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AC3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AF3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AH3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AI3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AK3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AN3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AO3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AP3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AQ3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AR3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AS3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AT3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AU3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AV3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AW3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="AX3" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="XEZ3" s="13"/>
-      <c r="XFA3" s="13"/>
-      <c r="XFB3" s="13"/>
-      <c r="XFC3" s="13"/>
-      <c r="XFD3" s="13"/>
+      <c r="BA2" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="BB2" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="BC2" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="BD2" s="14"/>
+      <c r="BE2" s="14"/>
+    </row>
+    <row r="3" s="23" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="J3" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="L3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="M3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="N3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="O3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="P3" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="R3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="S3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="T3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="U3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="V3" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="W3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="X3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="Y3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="Z3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AB3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AC3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AD3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AE3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AF3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AG3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AH3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AI3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AJ3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AL3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AM3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AO3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AP3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AQ3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AR3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AS3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AT3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AU3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AV3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AW3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AX3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AY3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="AZ3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="BA3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="BB3" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="BC3" s="25" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="C4" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="E4" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="F4" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="G4" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="B4" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="C4" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="J4" s="24" t="s">
+      <c r="D4" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="K4" s="24" t="s">
+      <c r="E4" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="L4" s="24" t="s">
+      <c r="F4" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="M4" s="24" t="s">
+      <c r="G4" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="N4" s="24" t="s">
+      <c r="H4" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="O4" s="24" t="s">
+      <c r="I4" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="P4" s="24" t="s">
+      <c r="J4" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="Q4" s="24" t="s">
+      <c r="K4" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="R4" s="24" t="s">
+      <c r="L4" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="S4" s="24" t="s">
+      <c r="M4" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="T4" s="24" t="s">
+      <c r="N4" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="U4" s="24" t="s">
+      <c r="O4" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="V4" s="24" t="s">
+      <c r="P4" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="W4" s="24" t="s">
+      <c r="Q4" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="X4" s="24" t="s">
+      <c r="R4" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="Y4" s="24" t="s">
+      <c r="S4" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="Z4" s="24" t="s">
+      <c r="T4" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="AA4" s="24" t="s">
+      <c r="U4" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="AB4" s="24" t="s">
+      <c r="V4" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="AC4" s="24" t="s">
+      <c r="W4" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="AD4" s="24" t="s">
+      <c r="X4" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="AE4" s="24" t="s">
+      <c r="Y4" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="AF4" s="24" t="s">
+      <c r="Z4" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="AG4" s="24" t="s">
+      <c r="AA4" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="AH4" s="24" t="s">
+      <c r="AB4" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="AI4" s="24" t="s">
+      <c r="AC4" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="AJ4" s="24" t="s">
+      <c r="AD4" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="AK4" s="24" t="s">
+      <c r="AE4" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="AL4" s="24" t="s">
+      <c r="AF4" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="AM4" s="24" t="s">
+      <c r="AG4" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="AN4" s="24" t="s">
+      <c r="AH4" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="AO4" s="24" t="s">
+      <c r="AI4" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="AP4" s="24" t="s">
+      <c r="AJ4" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="AQ4" s="24" t="s">
+      <c r="AK4" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="AR4" s="24" t="s">
+      <c r="AL4" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="AS4" s="24" t="s">
+      <c r="AM4" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="AT4" s="24" t="s">
+      <c r="AN4" s="26" t="s">
         <v>106</v>
       </c>
-      <c r="AU4" s="25" t="s">
+      <c r="AO4" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="AV4" s="25" t="s">
+      <c r="AP4" s="26" t="s">
         <v>108</v>
       </c>
+      <c r="AQ4" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="AR4" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="AS4" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="AT4" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="AU4" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="AV4" s="26" t="s">
+        <v>114</v>
+      </c>
       <c r="AW4" s="26" t="s">
-        <v>109</v>
-      </c>
-      <c r="AX4" s="27" t="s">
-        <v>110</v>
+        <v>115</v>
+      </c>
+      <c r="AX4" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="AY4" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="AZ4" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="BA4" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="BB4" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="BC4" s="29" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>5901234123457</v>
       </c>
-      <c r="G5" s="28" t="n">
+      <c r="G5" s="30" t="n">
         <v>45658</v>
       </c>
-      <c r="H5" s="28" t="s">
-        <v>116</v>
+      <c r="H5" s="30" t="s">
+        <v>127</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="J5" s="29" t="s">
-        <v>118</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="N5" s="28" t="s">
-        <v>121</v>
-      </c>
-      <c r="O5" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="P5" s="1" t="n">
+        <v>128</v>
+      </c>
+      <c r="J5" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="K5" s="31" t="s">
+        <v>130</v>
+      </c>
+      <c r="L5" s="31" t="s">
+        <v>131</v>
+      </c>
+      <c r="M5" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="N5" s="31" t="s">
+        <v>133</v>
+      </c>
+      <c r="O5" s="31"/>
+      <c r="P5" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="S5" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="T5" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="U5" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="Q5" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="T5" s="1" t="n">
+      <c r="V5" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="X5" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="Y5" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="U5" s="1" t="n">
+      <c r="Z5" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="V5" s="1" t="n">
+      <c r="AA5" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="W5" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="X5" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="Y5" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="Z5" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="AA5" s="1" t="n">
+      <c r="AB5" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="AC5" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="AD5" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="AE5" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="AF5" s="1" t="n">
         <v>0.385</v>
       </c>
-      <c r="AB5" s="1" t="n">
+      <c r="AG5" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="AC5" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="AD5" s="1" t="n">
+      <c r="AH5" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="AI5" s="1" t="n">
         <v>385</v>
       </c>
-      <c r="AE5" s="1" t="n">
+      <c r="AJ5" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="AF5" s="1" t="n">
+      <c r="AK5" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="AG5" s="28" t="s">
-        <v>128</v>
-      </c>
-      <c r="AH5" s="1" t="n">
+      <c r="AL5" s="30" t="s">
+        <v>143</v>
+      </c>
+      <c r="AM5" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="AI5" s="1" t="n">
+      <c r="AN5" s="1" t="n">
         <v>701000</v>
       </c>
-      <c r="AJ5" s="1" t="n">
+      <c r="AO5" s="1" t="n">
         <v>601000</v>
       </c>
-      <c r="AK5" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="AL5" s="1" t="s">
+      <c r="AP5" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="AM5" s="1" t="n">
+      <c r="AQ5" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="AR5" s="1" t="n">
         <v>84717050</v>
       </c>
-      <c r="AN5" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="AO5" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="AP5" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="AQ5" s="14" t="n">
+      <c r="AS5" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="AT5" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="AU5" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="AV5" s="15" t="n">
         <v>50.99</v>
       </c>
-      <c r="AR5" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="AS5" s="14" t="n">
+      <c r="AW5" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="AX5" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="AT5" s="14" t="n">
+      <c r="AY5" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="AU5" s="14" t="n">
+      <c r="AZ5" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="AV5" s="14" t="n">
+      <c r="BA5" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="AW5" s="28" t="n">
+      <c r="BB5" s="30" t="n">
         <v>45658</v>
       </c>
-      <c r="AX5" s="28" t="n">
+      <c r="BC5" s="30" t="n">
         <v>46022</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="AG6" s="30"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AL6" s="32"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2469,170 +2696,170 @@
   <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="16.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="15.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="26.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="16.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="31" width="24.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="31" width="11.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="31" width="9.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="31" width="17.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="31" width="10.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="31" width="16.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="31" width="17.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="31" width="11.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="31" width="11.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="33" width="16.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="33" width="15.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="33" width="26.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="33" width="16.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="33" width="24.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="33" width="11.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="33" width="9.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="33" width="17.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="33" width="10.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="33" width="16.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="33" width="17.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="33" width="11.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="33" width="11.08"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="18" min="14" style="1" width="10.16"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="20" style="31" width="10.16"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="20" style="33" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="B1" s="20" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="D1" s="20" t="s">
-        <v>137</v>
-      </c>
-      <c r="E1" s="20" t="s">
-        <v>135</v>
-      </c>
-      <c r="F1" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="G1" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="H1" s="20" t="s">
-        <v>138</v>
-      </c>
-      <c r="I1" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="J1" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="K1" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="L1" s="20" t="s">
+      <c r="A1" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="F1" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="M1" s="20" t="s">
-        <v>57</v>
+      <c r="G1" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="I1" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="J1" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="K1" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="L1" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="M1" s="22" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="B2" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="F2" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="G2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="H2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="I2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="J2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="K2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="L2" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="M2" s="23" t="s">
-        <v>60</v>
+      <c r="A2" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="H2" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="I2" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="K2" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="L2" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" s="25" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="32" t="s">
-        <v>139</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>140</v>
-      </c>
-      <c r="C3" s="33" t="s">
-        <v>141</v>
-      </c>
-      <c r="D3" s="32" t="s">
-        <v>142</v>
-      </c>
-      <c r="E3" s="32" t="s">
-        <v>143</v>
-      </c>
-      <c r="F3" s="32" t="s">
-        <v>144</v>
-      </c>
-      <c r="G3" s="32" t="s">
-        <v>145</v>
-      </c>
-      <c r="H3" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="I3" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="J3" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="K3" s="32" t="s">
-        <v>148</v>
-      </c>
-      <c r="L3" s="32" t="s">
-        <v>149</v>
-      </c>
-      <c r="M3" s="33" t="s">
-        <v>150</v>
+      <c r="A3" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="B3" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>156</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>158</v>
+      </c>
+      <c r="F3" s="34" t="s">
+        <v>159</v>
+      </c>
+      <c r="G3" s="34" t="s">
+        <v>160</v>
+      </c>
+      <c r="H3" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="I3" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="J3" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="K3" s="34" t="s">
+        <v>163</v>
+      </c>
+      <c r="L3" s="34" t="s">
+        <v>164</v>
+      </c>
+      <c r="M3" s="35" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>151</v>
+        <v>166</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>154</v>
+        <v>169</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>10</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="I4" s="1" t="n">
         <v>2</v>
@@ -2640,13 +2867,13 @@
       <c r="J4" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="K4" s="31" t="n">
+      <c r="K4" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="L4" s="28" t="n">
+      <c r="L4" s="30" t="n">
         <v>45658</v>
       </c>
-      <c r="M4" s="28" t="n">
+      <c r="M4" s="30" t="n">
         <v>46022</v>
       </c>
     </row>
@@ -2669,37 +2896,37 @@
   <dimension ref="A1:E1048576"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="34" width="27.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="35" width="102.88"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="3" style="36" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="36" width="27.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="37" width="102.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="3" style="38" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="37" t="s">
-        <v>158</v>
-      </c>
-      <c r="B1" s="37" t="s">
-        <v>159</v>
+      <c r="A1" s="39" t="s">
+        <v>173</v>
+      </c>
+      <c r="B1" s="39" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="195.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="38" t="s">
-        <v>160</v>
-      </c>
-      <c r="B2" s="38"/>
-    </row>
-    <row r="3" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="39"/>
-    </row>
-    <row r="4" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="39"/>
+      <c r="A2" s="40" t="s">
+        <v>175</v>
+      </c>
+      <c r="B2" s="40"/>
+    </row>
+    <row r="3" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="41"/>
+    </row>
+    <row r="4" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="41"/>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="40" t="s">
-        <v>159</v>
-      </c>
-      <c r="B5" s="41" t="s">
-        <v>161</v>
+      <c r="A5" s="42" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5" s="43" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2709,561 +2936,597 @@
       <c r="B6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="B7" s="36" t="s">
-        <v>162</v>
+      <c r="A7" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="38" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="B8" s="42" t="s">
-        <v>163</v>
+      <c r="A8" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="44" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="B9" s="42" t="s">
-        <v>164</v>
+      <c r="A9" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" s="42" t="s">
-        <v>165</v>
-      </c>
-      <c r="D10" s="34"/>
-      <c r="E10" s="42"/>
+      <c r="A10" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="44" t="s">
+        <v>180</v>
+      </c>
+      <c r="D10" s="36"/>
+      <c r="E10" s="44"/>
     </row>
     <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="B11" s="42" t="s">
-        <v>166</v>
+      <c r="A11" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="B12" s="42" t="s">
-        <v>167</v>
+      <c r="A12" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="44" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="B13" s="42" t="s">
-        <v>168</v>
+      <c r="A13" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="44" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="B14" s="42" t="s">
-        <v>169</v>
+      <c r="A14" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="B15" s="42" t="s">
-        <v>170</v>
+      <c r="A15" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="44" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25"/>
-      <c r="B16" s="42"/>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="43" t="s">
+      <c r="A16" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B17" s="43"/>
-    </row>
-    <row r="18" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="B18" s="42" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
-        <v>72</v>
-      </c>
-      <c r="B19" s="42" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="B20" s="42" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="B21" s="42" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="B22" s="42" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="B23" s="42" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="B16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="31.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="45" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="44" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="92.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="45" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" s="44" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="45" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="44" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="16.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="45" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="44" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="45" t="s">
+        <v>81</v>
+      </c>
+      <c r="B21" s="44"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="B24" s="5"/>
-    </row>
-    <row r="25" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="B25" s="42" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="B26" s="42" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="B27" s="42" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
+      <c r="B22" s="46"/>
+    </row>
+    <row r="23" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="44" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="44" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="44" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" s="44" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" s="44" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="B28" s="44" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="44"/>
-    </row>
-    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="B29" s="42" t="s">
-        <v>179</v>
-      </c>
+      <c r="B29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="25" t="s">
-        <v>81</v>
-      </c>
-      <c r="B30" s="42" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="B31" s="42" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="B32" s="42" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25" t="s">
-        <v>84</v>
-      </c>
-      <c r="B33" s="42" t="s">
-        <v>183</v>
-      </c>
+      <c r="A30" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" s="44" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="B31" s="44" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="B32" s="44" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="47"/>
     </row>
     <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="45" t="s">
-        <v>85</v>
-      </c>
-      <c r="B34" s="42" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="45" t="s">
-        <v>86</v>
-      </c>
-      <c r="B35" s="42" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B36" s="44"/>
-    </row>
-    <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="B37" s="42" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="B38" s="42" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="B34" s="44" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="B35" s="44" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" s="44" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B37" s="44" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" s="44" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="45" t="s">
-        <v>89</v>
-      </c>
-      <c r="B39" s="42" t="s">
-        <v>187</v>
+        <v>96</v>
+      </c>
+      <c r="B39" s="44" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="45" t="s">
-        <v>90</v>
-      </c>
-      <c r="B40" s="42" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="45" t="s">
-        <v>91</v>
-      </c>
-      <c r="B41" s="42" t="s">
-        <v>38</v>
-      </c>
+        <v>97</v>
+      </c>
+      <c r="B40" s="44" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B41" s="47"/>
     </row>
     <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="45" t="s">
-        <v>92</v>
-      </c>
-      <c r="B42" s="42" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="46" t="s">
-        <v>5</v>
-      </c>
-      <c r="B43" s="46"/>
-    </row>
-    <row r="44" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="B44" s="42" t="s">
-        <v>189</v>
-      </c>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-    </row>
-    <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="B45" s="42" t="s">
-        <v>190</v>
+      <c r="A42" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="B42" s="44" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="B43" s="44" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="45" t="s">
+        <v>100</v>
+      </c>
+      <c r="B44" s="44" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="B45" s="44" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="B46" s="42" t="s">
-        <v>191</v>
+      <c r="A46" s="45" t="s">
+        <v>102</v>
+      </c>
+      <c r="B46" s="44" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="B47" s="42" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="B48" s="42" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="47" t="s">
-        <v>194</v>
-      </c>
-      <c r="B49" s="47"/>
+      <c r="A47" s="45" t="s">
+        <v>103</v>
+      </c>
+      <c r="B47" s="44" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="48" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" s="48"/>
+    </row>
+    <row r="49" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="B49" s="44" t="s">
+        <v>207</v>
+      </c>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
     </row>
     <row r="50" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="27" t="s">
-        <v>98</v>
-      </c>
-      <c r="B50" s="42" t="s">
-        <v>195</v>
+        <v>105</v>
+      </c>
+      <c r="B50" s="44" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="B51" s="42" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="46.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="48" t="s">
-        <v>197</v>
-      </c>
-      <c r="B52" s="48"/>
+        <v>106</v>
+      </c>
+      <c r="B51" s="44" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B52" s="44" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="B53" s="42" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="B54" s="49" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="B55" s="49" t="s">
-        <v>200</v>
+      <c r="A53" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="B53" s="44" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="49" t="s">
+        <v>212</v>
+      </c>
+      <c r="B54" s="49"/>
+    </row>
+    <row r="55" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="29" t="s">
+        <v>109</v>
+      </c>
+      <c r="B55" s="44" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="B56" s="49" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="B57" s="49" t="s">
-        <v>202</v>
-      </c>
+      <c r="A56" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="B56" s="44" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="46.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="50" t="s">
+        <v>215</v>
+      </c>
+      <c r="B57" s="50"/>
     </row>
     <row r="58" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="B58" s="49" t="s">
-        <v>203</v>
+      <c r="A58" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B58" s="44" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="B59" s="42" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="B60" s="42" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="25" t="s">
-        <v>108</v>
-      </c>
-      <c r="B61" s="42" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="50" t="s">
-        <v>109</v>
+      <c r="A59" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="B59" s="51" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B60" s="51" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="B61" s="51" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="27" t="s">
+        <v>115</v>
       </c>
       <c r="B62" s="51" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="27" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B63" s="51" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B64" s="34"/>
-    </row>
-    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="34"/>
-    </row>
-    <row r="69" customFormat="false" ht="31.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="48" t="s">
-        <v>209</v>
-      </c>
-      <c r="B69" s="48"/>
-    </row>
-    <row r="70" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="25" t="s">
-        <v>139</v>
-      </c>
-      <c r="B70" s="42" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="27" t="s">
-        <v>140</v>
-      </c>
-      <c r="B71" s="42" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="B72" s="42" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="25" t="s">
-        <v>146</v>
-      </c>
-      <c r="B73" s="36" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="25" t="s">
-        <v>147</v>
-      </c>
-      <c r="B74" s="49" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="25" t="s">
-        <v>108</v>
-      </c>
-      <c r="B75" s="49"/>
-    </row>
-    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="50" t="s">
-        <v>148</v>
-      </c>
-      <c r="B76" s="49"/>
-    </row>
-    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="25" t="s">
-        <v>143</v>
-      </c>
-      <c r="B77" s="49"/>
+        <v>221</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="B64" s="44" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="B65" s="44" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="B66" s="44" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="52" t="s">
+        <v>120</v>
+      </c>
+      <c r="B67" s="53" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="B68" s="53" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="36"/>
+    </row>
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="36"/>
+    </row>
+    <row r="74" customFormat="false" ht="31.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="50" t="s">
+        <v>227</v>
+      </c>
+      <c r="B74" s="50"/>
+    </row>
+    <row r="75" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="27" t="s">
+        <v>154</v>
+      </c>
+      <c r="B75" s="44" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="B76" s="44" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="29" t="s">
+        <v>156</v>
+      </c>
+      <c r="B77" s="44" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="B78" s="49"/>
-    </row>
-    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="B79" s="49"/>
+      <c r="A78" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="B78" s="38" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="B79" s="51" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="25" t="s">
-        <v>145</v>
-      </c>
-      <c r="B80" s="49"/>
+      <c r="A80" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="B80" s="51"/>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="50" t="s">
-        <v>149</v>
-      </c>
-      <c r="B81" s="49"/>
-    </row>
-    <row r="82" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="52" t="s">
+        <v>163</v>
+      </c>
+      <c r="B81" s="51"/>
+    </row>
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="B82" s="49"/>
-    </row>
-    <row r="83" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="84" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="85" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="86" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="87" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="88" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="89" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="90" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="91" s="36" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>158</v>
+      </c>
+      <c r="B82" s="51"/>
+    </row>
+    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="B83" s="51"/>
+    </row>
+    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="B84" s="51"/>
+    </row>
+    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="B85" s="51"/>
+    </row>
+    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="52" t="s">
+        <v>164</v>
+      </c>
+      <c r="B86" s="51"/>
+    </row>
+    <row r="87" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="B87" s="51"/>
+    </row>
+    <row r="88" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="89" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="90" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="91" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="92" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="93" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="94" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="95" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="96" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -3271,16 +3534,16 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="B74:B82"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="B79:B87"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B51" r:id="rId1" display="Harmonized System Code.&#10;Est généralement configuré sur la famille d’article, et peut être redéfini par le HS Code du produit qui est plus prioritaire. Voir la nomenclature du World Customs Organisation : http://www.wcoomd.org/."/>
+    <hyperlink ref="B56" r:id="rId1" display="Harmonized System Code.&#10;Est généralement configuré sur la famille d’article, et peut être redéfini par le HS Code du produit qui est plus prioritaire. Voir la nomenclature du World Customs Organisation : http://www.wcoomd.org/."/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[IMP] - add support of a method to import variant: fixed price, 1 line of the file = 1 variant - add support of category code - fix logs not showing for products
</commit_message>
<xml_diff>
--- a/product_import_helper/static/xls/product_import_helper_template.xlsx
+++ b/product_import_helper/static/xls/product_import_helper_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" state="visible" r:id="rId3"/>
@@ -255,7 +255,7 @@
     <t xml:space="preserve">is_storable</t>
   </si>
   <si>
-    <t xml:space="preserve">default_code_tmpl</t>
+    <t xml:space="preserve">pivot_code_tmpl</t>
   </si>
   <si>
     <t xml:space="preserve">attr_Name1</t>
@@ -599,7 +599,27 @@
 L’import alerte concernant les doublons.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nom de la famille d’article. Si le nom correspond exactement à une catégorie existante (hormis la casse), elle sera réutilisée et lié à l’article. Si le nom est inconnu, elle sera créée.</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Code ou nom de la famille d’article :
+- s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">i le code ou le nom de la famille d’article est inconnu en base, elle sera créée
+- sinon, elle sera retrouvée et définie sur l’article</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Idem, pour le point de vente. Si pas installé, supprimer la colonne.</t>
@@ -627,12 +647,12 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Si renseigné, l’import bascule en mode “gestion des variants” et la référence </t>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Si renseigné, l’import bascule en mode “gestion des variants” et la clef </t>
     </r>
     <r>
       <rPr>
@@ -643,17 +663,105 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">default_code_tmpl</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> désigne la référence de l’article de base (le “template”).</t>
+      <t xml:space="preserve">pivot_code_tmpl </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">doit être renseignée. Sa valeur doit être identique entre tous les variants d’un même modèle article (product.template) pour que le mécanisme d’import sache rattacher les variants entre eux.
+La valeur renseignée peut être :
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">la référence d’un variant déjà existant en base</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> : le système d’import retrouvera le modèle d’article (product.template) lié
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">pour un import dans une base vide </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: simplement une clef commune à tous les variants. Ce peut être un nombre, la référence du 1</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">er</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> variant importé, ou bien la référence épurée des variants.
+Exemple : pour 2 variants aux références « Paumelle-vert » et « Paumelle-bleu », le </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">pivot_code_tmpl</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> peut être « Paumelle »</t>
     </r>
   </si>
   <si>
@@ -1193,9 +1301,9 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
+    <numFmt numFmtId="166" formatCode="&quot;VRAI&quot;;&quot;VRAI&quot;;&quot;FAUX&quot;"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1306,6 +1414,28 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <vertAlign val="superscript"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <u val="single"/>
       <sz val="11"/>
       <color theme="1"/>
@@ -1410,7 +1540,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1595,6 +1725,10 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1615,7 +1749,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2951,7 +3085,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="46.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
         <v>69</v>
       </c>
@@ -3015,15 +3149,15 @@
       </c>
       <c r="B16" s="4"/>
     </row>
-    <row r="17" customFormat="false" ht="31.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="165.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="45" t="s">
         <v>77</v>
       </c>
-      <c r="B17" s="44" t="s">
+      <c r="B17" s="46" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="92.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="45" t="s">
         <v>78</v>
       </c>
@@ -3039,7 +3173,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="45" t="s">
         <v>80</v>
       </c>
@@ -3054,10 +3188,10 @@
       <c r="B21" s="44"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="46" t="s">
+      <c r="A22" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B22" s="46"/>
+      <c r="B22" s="47"/>
     </row>
     <row r="23" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="27" t="s">
@@ -3141,7 +3275,7 @@
       <c r="A33" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B33" s="47"/>
+      <c r="B33" s="48"/>
     </row>
     <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="27" t="s">
@@ -3203,7 +3337,7 @@
       <c r="A41" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B41" s="47"/>
+      <c r="B41" s="48"/>
     </row>
     <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="27" t="s">
@@ -3254,10 +3388,10 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="48" t="s">
+      <c r="A48" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="B48" s="48"/>
+      <c r="B48" s="49"/>
     </row>
     <row r="49" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="27" t="s">
@@ -3303,10 +3437,10 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="49" t="s">
+      <c r="A54" s="50" t="s">
         <v>212</v>
       </c>
-      <c r="B54" s="49"/>
+      <c r="B54" s="50"/>
     </row>
     <row r="55" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="29" t="s">
@@ -3325,10 +3459,10 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="46.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="50" t="s">
+      <c r="A57" s="51" t="s">
         <v>215</v>
       </c>
-      <c r="B57" s="50"/>
+      <c r="B57" s="51"/>
     </row>
     <row r="58" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="27" t="s">
@@ -3342,7 +3476,7 @@
       <c r="A59" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="B59" s="51" t="s">
+      <c r="B59" s="52" t="s">
         <v>217</v>
       </c>
     </row>
@@ -3350,7 +3484,7 @@
       <c r="A60" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="B60" s="51" t="s">
+      <c r="B60" s="52" t="s">
         <v>218</v>
       </c>
     </row>
@@ -3358,7 +3492,7 @@
       <c r="A61" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="B61" s="51" t="s">
+      <c r="B61" s="52" t="s">
         <v>219</v>
       </c>
     </row>
@@ -3366,7 +3500,7 @@
       <c r="A62" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="B62" s="51" t="s">
+      <c r="B62" s="52" t="s">
         <v>220</v>
       </c>
     </row>
@@ -3374,7 +3508,7 @@
       <c r="A63" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="B63" s="51" t="s">
+      <c r="B63" s="52" t="s">
         <v>221</v>
       </c>
     </row>
@@ -3403,10 +3537,10 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="52" t="s">
+      <c r="A67" s="53" t="s">
         <v>120</v>
       </c>
-      <c r="B67" s="53" t="s">
+      <c r="B67" s="54" t="s">
         <v>225</v>
       </c>
     </row>
@@ -3414,7 +3548,7 @@
       <c r="A68" s="29" t="s">
         <v>121</v>
       </c>
-      <c r="B68" s="53" t="s">
+      <c r="B68" s="54" t="s">
         <v>226</v>
       </c>
     </row>
@@ -3425,10 +3559,10 @@
       <c r="B70" s="36"/>
     </row>
     <row r="74" customFormat="false" ht="31.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="50" t="s">
+      <c r="A74" s="51" t="s">
         <v>227</v>
       </c>
-      <c r="B74" s="50"/>
+      <c r="B74" s="51"/>
     </row>
     <row r="75" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="27" t="s">
@@ -3466,7 +3600,7 @@
       <c r="A79" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="B79" s="51" t="s">
+      <c r="B79" s="52" t="s">
         <v>232</v>
       </c>
     </row>
@@ -3474,49 +3608,49 @@
       <c r="A80" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="B80" s="51"/>
+      <c r="B80" s="52"/>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="52" t="s">
+      <c r="A81" s="53" t="s">
         <v>163</v>
       </c>
-      <c r="B81" s="51"/>
+      <c r="B81" s="52"/>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="27" t="s">
         <v>158</v>
       </c>
-      <c r="B82" s="51"/>
+      <c r="B82" s="52"/>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="B83" s="51"/>
+      <c r="B83" s="52"/>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="27" t="s">
         <v>159</v>
       </c>
-      <c r="B84" s="51"/>
+      <c r="B84" s="52"/>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="B85" s="51"/>
+      <c r="B85" s="52"/>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="52" t="s">
+      <c r="A86" s="53" t="s">
         <v>164</v>
       </c>
-      <c r="B86" s="51"/>
+      <c r="B86" s="52"/>
     </row>
     <row r="87" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="B87" s="51"/>
+      <c r="B87" s="52"/>
     </row>
     <row r="88" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="89" s="38" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
[FIX] little issue "ValueError: Invalid field 'tags' on model 'product.product'"
</commit_message>
<xml_diff>
--- a/product_import_helper/static/xls/product_import_helper_template.xlsx
+++ b/product_import_helper/static/xls/product_import_helper_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" state="visible" r:id="rId3"/>
@@ -599,27 +599,9 @@
 L’import alerte concernant les doublons.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Code ou nom de la famille d’article :
-- s</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">i le code ou le nom de la famille d’article est inconnu en base, elle sera créée
+    <t xml:space="preserve">Code ou nom de la famille d’article :
+- si le code ou le nom de la famille d’article est inconnu en base, elle sera créée
 - sinon, elle sera retrouvée et définie sur l’article</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">Idem, pour le point de vente. Si pas installé, supprimer la colonne.</t>
@@ -1303,7 +1285,7 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="&quot;VRAI&quot;;&quot;VRAI&quot;;&quot;FAUX&quot;"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1414,12 +1396,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
-    <font>
       <u val="single"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1749,7 +1725,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3085,7 +3061,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="46.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
         <v>69</v>
       </c>

</xml_diff>

<commit_message>
[FIX] product_import_helpler: in .xlsx template, rename 'list_price' by 'lst_price' to be compatible with 'product_variant_sale_price'
</commit_message>
<xml_diff>
--- a/product_import_helper/static/xls/product_import_helper_template.xlsx
+++ b/product_import_helper/static/xls/product_import_helper_template.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="234">
   <si>
     <t xml:space="preserve">IDENTIFICATION</t>
   </si>
@@ -276,7 +276,7 @@
     <t xml:space="preserve">invoice_policy</t>
   </si>
   <si>
-    <t xml:space="preserve">list_price</t>
+    <t xml:space="preserve">lst_price</t>
   </si>
   <si>
     <t xml:space="preserve">tags</t>
@@ -885,6 +885,9 @@
       </rPr>
       <t xml:space="preserve"> : facturer sur base des quantites livrées au client.</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">list_price</t>
   </si>
   <si>
     <t xml:space="preserve">Prix de vente.</t>
@@ -3187,10 +3190,10 @@
     </row>
     <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="27" t="s">
-        <v>84</v>
+        <v>191</v>
       </c>
       <c r="B25" s="44" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3206,7 +3209,7 @@
         <v>86</v>
       </c>
       <c r="B27" s="44" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3214,7 +3217,7 @@
         <v>87</v>
       </c>
       <c r="B28" s="44" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3228,7 +3231,7 @@
         <v>88</v>
       </c>
       <c r="B30" s="44" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3236,7 +3239,7 @@
         <v>89</v>
       </c>
       <c r="B31" s="44" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3244,7 +3247,7 @@
         <v>90</v>
       </c>
       <c r="B32" s="44" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3258,7 +3261,7 @@
         <v>91</v>
       </c>
       <c r="B34" s="44" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3266,7 +3269,7 @@
         <v>92</v>
       </c>
       <c r="B35" s="44" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3274,7 +3277,7 @@
         <v>93</v>
       </c>
       <c r="B36" s="44" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3282,7 +3285,7 @@
         <v>94</v>
       </c>
       <c r="B37" s="44" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3290,7 +3293,7 @@
         <v>95</v>
       </c>
       <c r="B38" s="44" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3298,7 +3301,7 @@
         <v>96</v>
       </c>
       <c r="B39" s="44" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3306,7 +3309,7 @@
         <v>97</v>
       </c>
       <c r="B40" s="44" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3328,7 +3331,7 @@
         <v>99</v>
       </c>
       <c r="B43" s="44" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3336,7 +3339,7 @@
         <v>100</v>
       </c>
       <c r="B44" s="44" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3344,7 +3347,7 @@
         <v>101</v>
       </c>
       <c r="B45" s="44" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3374,7 +3377,7 @@
         <v>104</v>
       </c>
       <c r="B49" s="44" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C49" s="14"/>
       <c r="D49" s="14"/>
@@ -3385,7 +3388,7 @@
         <v>105</v>
       </c>
       <c r="B50" s="44" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3393,7 +3396,7 @@
         <v>106</v>
       </c>
       <c r="B51" s="44" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3401,7 +3404,7 @@
         <v>107</v>
       </c>
       <c r="B52" s="44" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3409,12 +3412,12 @@
         <v>108</v>
       </c>
       <c r="B53" s="44" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="50" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B54" s="50"/>
     </row>
@@ -3423,7 +3426,7 @@
         <v>109</v>
       </c>
       <c r="B55" s="44" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3431,12 +3434,12 @@
         <v>110</v>
       </c>
       <c r="B56" s="44" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="46.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="51" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B57" s="51"/>
     </row>
@@ -3445,7 +3448,7 @@
         <v>111</v>
       </c>
       <c r="B58" s="44" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3453,7 +3456,7 @@
         <v>112</v>
       </c>
       <c r="B59" s="52" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3461,7 +3464,7 @@
         <v>113</v>
       </c>
       <c r="B60" s="52" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3469,7 +3472,7 @@
         <v>114</v>
       </c>
       <c r="B61" s="52" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3477,7 +3480,7 @@
         <v>115</v>
       </c>
       <c r="B62" s="52" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3485,7 +3488,7 @@
         <v>116</v>
       </c>
       <c r="B63" s="52" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3493,7 +3496,7 @@
         <v>117</v>
       </c>
       <c r="B64" s="44" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3501,7 +3504,7 @@
         <v>118</v>
       </c>
       <c r="B65" s="44" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3509,7 +3512,7 @@
         <v>119</v>
       </c>
       <c r="B66" s="44" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3517,7 +3520,7 @@
         <v>120</v>
       </c>
       <c r="B67" s="54" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3525,7 +3528,7 @@
         <v>121</v>
       </c>
       <c r="B68" s="54" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3536,7 +3539,7 @@
     </row>
     <row r="74" customFormat="false" ht="31.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="51" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B74" s="51"/>
     </row>
@@ -3545,7 +3548,7 @@
         <v>154</v>
       </c>
       <c r="B75" s="44" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3553,7 +3556,7 @@
         <v>155</v>
       </c>
       <c r="B76" s="44" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3561,7 +3564,7 @@
         <v>156</v>
       </c>
       <c r="B77" s="44" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3569,7 +3572,7 @@
         <v>161</v>
       </c>
       <c r="B78" s="38" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3577,7 +3580,7 @@
         <v>162</v>
       </c>
       <c r="B79" s="52" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>